<commit_message>
fix(f4): use intakeYear/intakeSemester for year derivation; redesign MEDIUM test
- deriveStudentYear now prefers intakeYear+intakeSemester passed directly
  on the API body, avoiding DD/MM/YYYY date-parsing ambiguity that caused
  off-by-one year errors
- Fix assessFailedUnits and assessYearLevelGap to read missingUnits from
  primaryMajor.breakdown (DisplayPayload shape) instead of unmatchedCore
  which does not exist on the match payload
- MEDIUM test redesigned: COS30018 now grade F (still counted by matcher,
  flagged by assessFailedUnits at MEDIUM; no yearLevelGap fires)
- All 4 test transcripts regenerated to correctly target CRITICAL/HIGH/MEDIUM/LOW
</commit_message>
<xml_diff>
--- a/test-data/test-transcript-MEDIUM.xlsx
+++ b/test-data/test-transcript-MEDIUM.xlsx
@@ -409,7 +409,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G27"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -566,7 +566,7 @@
         <v>Complete</v>
       </c>
       <c r="F7" s="2" t="str">
-        <v>B</v>
+        <v>A-</v>
       </c>
       <c r="G7" s="2" t="str">
         <v>2024/S1</v>
@@ -589,7 +589,7 @@
         <v>Complete</v>
       </c>
       <c r="F8" s="2" t="str">
-        <v>B+</v>
+        <v>A</v>
       </c>
       <c r="G8" s="2" t="str">
         <v>2024/S1</v>
@@ -612,7 +612,7 @@
         <v>Complete</v>
       </c>
       <c r="F9" s="2" t="str">
-        <v>B</v>
+        <v>A-</v>
       </c>
       <c r="G9" s="2" t="str">
         <v>2024/S1</v>
@@ -620,22 +620,22 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="str">
-        <v>MPU3212</v>
+        <v>COS30015</v>
       </c>
       <c r="B10" s="2" t="str">
-        <v>Bahasa Kebangsaan A</v>
+        <v>IT Security</v>
       </c>
       <c r="C10" s="2">
-        <v>0</v>
+        <v>12.5</v>
       </c>
       <c r="D10" s="2">
-        <v>0</v>
+        <v>12.5</v>
       </c>
       <c r="E10" s="2" t="str">
         <v>Complete</v>
       </c>
       <c r="F10" s="2" t="str">
-        <v>Pass</v>
+        <v>B+</v>
       </c>
       <c r="G10" s="2" t="str">
         <v>2024/S1</v>
@@ -643,33 +643,33 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="str">
-        <v>COS20031</v>
+        <v>MPU3212</v>
       </c>
       <c r="B11" s="2" t="str">
-        <v>Database Design Project</v>
+        <v>Bahasa Kebangsaan A</v>
       </c>
       <c r="C11" s="2">
-        <v>12.5</v>
+        <v>0</v>
       </c>
       <c r="D11" s="2">
-        <v>12.5</v>
+        <v>0</v>
       </c>
       <c r="E11" s="2" t="str">
         <v>Complete</v>
       </c>
       <c r="F11" s="2" t="str">
-        <v>B</v>
+        <v>Pass</v>
       </c>
       <c r="G11" s="2" t="str">
-        <v>2024/S2</v>
+        <v>2024/S1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="str">
-        <v>COS30019</v>
+        <v>COS20031</v>
       </c>
       <c r="B12" s="2" t="str">
-        <v>Introduction to Artificial Intelligence</v>
+        <v>Database Design Project</v>
       </c>
       <c r="C12" s="2">
         <v>12.5</v>
@@ -681,7 +681,7 @@
         <v>Complete</v>
       </c>
       <c r="F12" s="2" t="str">
-        <v>B+</v>
+        <v>A-</v>
       </c>
       <c r="G12" s="2" t="str">
         <v>2024/S2</v>
@@ -689,10 +689,10 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="str">
-        <v>SWE30009</v>
+        <v>COS30019</v>
       </c>
       <c r="B13" s="2" t="str">
-        <v>Software Testing and Reliability</v>
+        <v>Introduction to Artificial Intelligence</v>
       </c>
       <c r="C13" s="2">
         <v>12.5</v>
@@ -704,7 +704,7 @@
         <v>Complete</v>
       </c>
       <c r="F13" s="2" t="str">
-        <v>C+</v>
+        <v>A</v>
       </c>
       <c r="G13" s="2" t="str">
         <v>2024/S2</v>
@@ -712,22 +712,22 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="str">
-        <v>MPU3143</v>
+        <v>SWE30009</v>
       </c>
       <c r="B14" s="2" t="str">
-        <v>Malay Language Communication 2</v>
+        <v>Software Testing and Reliability</v>
       </c>
       <c r="C14" s="2">
-        <v>0</v>
+        <v>12.5</v>
       </c>
       <c r="D14" s="2">
-        <v>0</v>
+        <v>12.5</v>
       </c>
       <c r="E14" s="2" t="str">
         <v>Complete</v>
       </c>
       <c r="F14" s="2" t="str">
-        <v>Pass</v>
+        <v>B+</v>
       </c>
       <c r="G14" s="2" t="str">
         <v>2024/S2</v>
@@ -735,10 +735,10 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="str">
-        <v>MPU3183</v>
+        <v>MPU3143</v>
       </c>
       <c r="B15" s="2" t="str">
-        <v>Penghayatan Etika dan Peradaban</v>
+        <v>Malay Language Communication 2</v>
       </c>
       <c r="C15" s="2">
         <v>0</v>
@@ -758,33 +758,33 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="str">
-        <v>COS10004</v>
+        <v>MPU3183</v>
       </c>
       <c r="B16" s="2" t="str">
-        <v>Computer Systems</v>
+        <v>Penghayatan Etika dan Peradaban</v>
       </c>
       <c r="C16" s="2">
-        <v>12.5</v>
+        <v>0</v>
       </c>
       <c r="D16" s="2">
-        <v>12.5</v>
+        <v>0</v>
       </c>
       <c r="E16" s="2" t="str">
         <v>Complete</v>
       </c>
       <c r="F16" s="2" t="str">
-        <v>B</v>
+        <v>Pass</v>
       </c>
       <c r="G16" s="2" t="str">
-        <v>2025/S1</v>
+        <v>2024/S2</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="str">
-        <v>COS20019</v>
+        <v>COS10004</v>
       </c>
       <c r="B17" s="2" t="str">
-        <v>Cloud Computing Architecture</v>
+        <v>Computer Systems</v>
       </c>
       <c r="C17" s="2">
         <v>12.5</v>
@@ -796,7 +796,7 @@
         <v>Complete</v>
       </c>
       <c r="F17" s="2" t="str">
-        <v>B-</v>
+        <v>A-</v>
       </c>
       <c r="G17" s="2" t="str">
         <v>2025/S1</v>
@@ -804,10 +804,10 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="str">
-        <v>COS30049</v>
+        <v>COS20019</v>
       </c>
       <c r="B18" s="2" t="str">
-        <v>Computing Technology Innovation Project</v>
+        <v>Cloud Computing Architecture</v>
       </c>
       <c r="C18" s="2">
         <v>12.5</v>
@@ -819,7 +819,7 @@
         <v>Complete</v>
       </c>
       <c r="F18" s="2" t="str">
-        <v>B</v>
+        <v>A</v>
       </c>
       <c r="G18" s="2" t="str">
         <v>2025/S1</v>
@@ -827,10 +827,10 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="str">
-        <v>COS40005</v>
+        <v>COS30018</v>
       </c>
       <c r="B19" s="2" t="str">
-        <v>Computing Technology Project A</v>
+        <v>Intelligent Systems</v>
       </c>
       <c r="C19" s="2">
         <v>12.5</v>
@@ -839,41 +839,202 @@
         <v>0</v>
       </c>
       <c r="E19" s="2" t="str">
-        <v>Current</v>
+        <v>Incomplete</v>
       </c>
       <c r="F19" s="2" t="str">
-        <v>N</v>
+        <v>F</v>
       </c>
       <c r="G19" s="2" t="str">
-        <v>2025/S2</v>
+        <v>2025/S1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="str">
+        <v>COS30049</v>
+      </c>
+      <c r="B20" s="2" t="str">
+        <v>Computing Technology Innovation Project</v>
+      </c>
+      <c r="C20" s="2">
+        <v>12.5</v>
+      </c>
+      <c r="D20" s="2">
+        <v>12.5</v>
+      </c>
+      <c r="E20" s="2" t="str">
+        <v>Complete</v>
+      </c>
+      <c r="F20" s="2" t="str">
+        <v>A-</v>
+      </c>
+      <c r="G20" s="2" t="str">
+        <v>2025/S1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="str">
+        <v>COS40005</v>
+      </c>
+      <c r="B21" s="2" t="str">
+        <v>Computing Technology Project A</v>
+      </c>
+      <c r="C21" s="2">
+        <v>12.5</v>
+      </c>
+      <c r="D21" s="2">
+        <v>12.5</v>
+      </c>
+      <c r="E21" s="2" t="str">
+        <v>Complete</v>
+      </c>
+      <c r="F21" s="2" t="str">
+        <v>A</v>
+      </c>
+      <c r="G21" s="2" t="str">
+        <v>2025/S2</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="str">
         <v>COS30082</v>
       </c>
-      <c r="B20" s="2" t="str">
+      <c r="B22" s="2" t="str">
         <v>Applied Machine Learning</v>
       </c>
-      <c r="C20" s="2">
-        <v>12.5</v>
-      </c>
-      <c r="D20" s="2">
-        <v>0</v>
-      </c>
-      <c r="E20" s="2" t="str">
+      <c r="C22" s="2">
+        <v>12.5</v>
+      </c>
+      <c r="D22" s="2">
+        <v>12.5</v>
+      </c>
+      <c r="E22" s="2" t="str">
+        <v>Complete</v>
+      </c>
+      <c r="F22" s="2" t="str">
+        <v>A</v>
+      </c>
+      <c r="G22" s="2" t="str">
+        <v>2025/S2</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="str">
+        <v>COS40006</v>
+      </c>
+      <c r="B23" s="2" t="str">
+        <v>Computing Technology Project B</v>
+      </c>
+      <c r="C23" s="2">
+        <v>12.5</v>
+      </c>
+      <c r="D23" s="2">
+        <v>0</v>
+      </c>
+      <c r="E23" s="2" t="str">
         <v>Current</v>
       </c>
-      <c r="F20" s="2" t="str">
+      <c r="F23" s="2" t="str">
         <v>N</v>
       </c>
-      <c r="G20" s="2" t="str">
+      <c r="G23" s="2" t="str">
+        <v>2026/S1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="str">
+        <v>COS40007</v>
+      </c>
+      <c r="B24" s="2" t="str">
+        <v>Artificial Intelligence for Engineering</v>
+      </c>
+      <c r="C24" s="2">
+        <v>12.5</v>
+      </c>
+      <c r="D24" s="2">
+        <v>0</v>
+      </c>
+      <c r="E24" s="2" t="str">
+        <v>Current</v>
+      </c>
+      <c r="F24" s="2" t="str">
+        <v>N</v>
+      </c>
+      <c r="G24" s="2" t="str">
+        <v>2026/S1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="str">
+        <v>SWE30003</v>
+      </c>
+      <c r="B25" s="2" t="str">
+        <v>Software Architecture and Design</v>
+      </c>
+      <c r="C25" s="2">
+        <v>12.5</v>
+      </c>
+      <c r="D25" s="2">
+        <v>0</v>
+      </c>
+      <c r="E25" s="2" t="str">
+        <v>Current</v>
+      </c>
+      <c r="F25" s="2" t="str">
+        <v>N</v>
+      </c>
+      <c r="G25" s="2" t="str">
+        <v>2026/S1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="str">
+        <v>COS20083</v>
+      </c>
+      <c r="B26" s="2" t="str">
+        <v>Advanced Data Analytics</v>
+      </c>
+      <c r="C26" s="2">
+        <v>12.5</v>
+      </c>
+      <c r="D26" s="2">
+        <v>12.5</v>
+      </c>
+      <c r="E26" s="2" t="str">
+        <v>Complete</v>
+      </c>
+      <c r="F26" s="2" t="str">
+        <v>B+</v>
+      </c>
+      <c r="G26" s="2" t="str">
+        <v>2025/S1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="str">
+        <v>COS30045</v>
+      </c>
+      <c r="B27" s="2" t="str">
+        <v>Data Visualisation</v>
+      </c>
+      <c r="C27" s="2">
+        <v>12.5</v>
+      </c>
+      <c r="D27" s="2">
+        <v>12.5</v>
+      </c>
+      <c r="E27" s="2" t="str">
+        <v>Complete</v>
+      </c>
+      <c r="F27" s="2" t="str">
+        <v>B</v>
+      </c>
+      <c r="G27" s="2" t="str">
         <v>2025/S2</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G27"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>